<commit_message>
Update PartyCode.xlsx from PO app
</commit_message>
<xml_diff>
--- a/PartyCode.xlsx
+++ b/PartyCode.xlsx
@@ -1,42 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30513"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\veraj\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3241E04D-0CA5-3541-8CDD-C9ADBBCDD9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86241B05-6681-462A-8486-9F0FAF9DC957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{99EBD75F-AF2A-43B3-9555-8F8B52E04ADC}"/>
   </bookViews>
   <sheets>
     <sheet name="ORB_PtyUPdateReport" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="536">
   <si>
     <t>Party Code</t>
   </si>
@@ -1644,9 +1633,6 @@
   </si>
   <si>
     <t>ZEPTO LIMITED - West Bengal</t>
-  </si>
-  <si>
-    <t>ZEPTO LIMITED - Coimbatore</t>
   </si>
 </sst>
 </file>
@@ -1753,9 +1739,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1793,7 +1779,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1899,7 +1885,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2041,7 +2027,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2049,17 +2035,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6EB0927-B5A6-4BE7-9AEA-68E6BA930412}">
-  <dimension ref="A1:E194"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E193"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.24609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.2578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="46.8125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.2578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2076,7 +2062,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -2093,7 +2079,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -2110,7 +2096,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -2127,7 +2113,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>31</v>
       </c>
@@ -2144,7 +2130,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>35</v>
       </c>
@@ -2161,7 +2147,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>39</v>
       </c>
@@ -2178,7 +2164,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>41</v>
       </c>
@@ -2195,7 +2181,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>44</v>
       </c>
@@ -2212,7 +2198,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>48</v>
       </c>
@@ -2229,7 +2215,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>51</v>
       </c>
@@ -2246,7 +2232,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>55</v>
       </c>
@@ -2263,7 +2249,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>58</v>
       </c>
@@ -2280,7 +2266,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>61</v>
       </c>
@@ -2297,7 +2283,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>65</v>
       </c>
@@ -2314,7 +2300,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>68</v>
       </c>
@@ -2331,7 +2317,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>71</v>
       </c>
@@ -2348,7 +2334,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>74</v>
       </c>
@@ -2365,7 +2351,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>77</v>
       </c>
@@ -2382,7 +2368,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>80</v>
       </c>
@@ -2399,7 +2385,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>83</v>
       </c>
@@ -2416,7 +2402,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>86</v>
       </c>
@@ -2433,7 +2419,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>89</v>
       </c>
@@ -2450,7 +2436,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>92</v>
       </c>
@@ -2467,7 +2453,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>95</v>
       </c>
@@ -2484,7 +2470,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>98</v>
       </c>
@@ -2501,7 +2487,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>101</v>
       </c>
@@ -2518,7 +2504,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>104</v>
       </c>
@@ -2535,7 +2521,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>107</v>
       </c>
@@ -2552,7 +2538,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>110</v>
       </c>
@@ -2569,7 +2555,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>113</v>
       </c>
@@ -2586,7 +2572,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>116</v>
       </c>
@@ -2603,7 +2589,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>119</v>
       </c>
@@ -2620,7 +2606,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>122</v>
       </c>
@@ -2637,7 +2623,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>125</v>
       </c>
@@ -2654,7 +2640,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>128</v>
       </c>
@@ -2671,7 +2657,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>131</v>
       </c>
@@ -2688,7 +2674,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>134</v>
       </c>
@@ -2705,7 +2691,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>137</v>
       </c>
@@ -2722,7 +2708,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>140</v>
       </c>
@@ -2739,7 +2725,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>143</v>
       </c>
@@ -2756,7 +2742,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>146</v>
       </c>
@@ -2773,7 +2759,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>149</v>
       </c>
@@ -2790,7 +2776,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>152</v>
       </c>
@@ -2807,7 +2793,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>154</v>
       </c>
@@ -2824,7 +2810,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>156</v>
       </c>
@@ -2841,7 +2827,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>159</v>
       </c>
@@ -2858,7 +2844,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>162</v>
       </c>
@@ -2875,7 +2861,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>165</v>
       </c>
@@ -2892,7 +2878,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>168</v>
       </c>
@@ -2909,7 +2895,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>170</v>
       </c>
@@ -2926,7 +2912,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>172</v>
       </c>
@@ -2943,7 +2929,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>176</v>
       </c>
@@ -2960,7 +2946,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>180</v>
       </c>
@@ -2977,7 +2963,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>183</v>
       </c>
@@ -2994,7 +2980,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>186</v>
       </c>
@@ -3011,7 +2997,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>189</v>
       </c>
@@ -3028,7 +3014,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>191</v>
       </c>
@@ -3045,7 +3031,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>193</v>
       </c>
@@ -3062,7 +3048,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>195</v>
       </c>
@@ -3079,7 +3065,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>199</v>
       </c>
@@ -3096,7 +3082,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>203</v>
       </c>
@@ -3113,7 +3099,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>206</v>
       </c>
@@ -3130,7 +3116,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>209</v>
       </c>
@@ -3147,7 +3133,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>212</v>
       </c>
@@ -3164,7 +3150,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>214</v>
       </c>
@@ -3181,7 +3167,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>217</v>
       </c>
@@ -3198,7 +3184,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>219</v>
       </c>
@@ -3215,7 +3201,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>221</v>
       </c>
@@ -3232,7 +3218,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>225</v>
       </c>
@@ -3249,7 +3235,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>228</v>
       </c>
@@ -3266,7 +3252,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>231</v>
       </c>
@@ -3283,7 +3269,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>233</v>
       </c>
@@ -3300,7 +3286,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>237</v>
       </c>
@@ -3317,7 +3303,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>240</v>
       </c>
@@ -3334,7 +3320,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>242</v>
       </c>
@@ -3351,7 +3337,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>245</v>
       </c>
@@ -3368,7 +3354,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>248</v>
       </c>
@@ -3385,7 +3371,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>251</v>
       </c>
@@ -3402,7 +3388,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>253</v>
       </c>
@@ -3419,7 +3405,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>255</v>
       </c>
@@ -3436,7 +3422,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>258</v>
       </c>
@@ -3453,7 +3439,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>261</v>
       </c>
@@ -3470,7 +3456,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>264</v>
       </c>
@@ -3487,7 +3473,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>267</v>
       </c>
@@ -3504,7 +3490,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>270</v>
       </c>
@@ -3521,7 +3507,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>273</v>
       </c>
@@ -3538,7 +3524,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>275</v>
       </c>
@@ -3555,7 +3541,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>277</v>
       </c>
@@ -3572,7 +3558,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>279</v>
       </c>
@@ -3589,7 +3575,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>282</v>
       </c>
@@ -3606,7 +3592,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>288</v>
       </c>
@@ -3623,7 +3609,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>291</v>
       </c>
@@ -3640,7 +3626,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>294</v>
       </c>
@@ -3657,7 +3643,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>297</v>
       </c>
@@ -3674,7 +3660,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>299</v>
       </c>
@@ -3691,7 +3677,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>302</v>
       </c>
@@ -3708,7 +3694,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>305</v>
       </c>
@@ -3725,7 +3711,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>308</v>
       </c>
@@ -3742,7 +3728,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>311</v>
       </c>
@@ -3759,7 +3745,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>313</v>
       </c>
@@ -3776,7 +3762,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>315</v>
       </c>
@@ -3793,7 +3779,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>317</v>
       </c>
@@ -3810,7 +3796,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>319</v>
       </c>
@@ -3827,7 +3813,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>322</v>
       </c>
@@ -3844,7 +3830,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>325</v>
       </c>
@@ -3861,7 +3847,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>328</v>
       </c>
@@ -3878,7 +3864,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>331</v>
       </c>
@@ -3895,7 +3881,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>334</v>
       </c>
@@ -3912,7 +3898,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>338</v>
       </c>
@@ -3929,7 +3915,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>341</v>
       </c>
@@ -3946,7 +3932,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>344</v>
       </c>
@@ -3963,7 +3949,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>346</v>
       </c>
@@ -3980,7 +3966,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>348</v>
       </c>
@@ -3997,7 +3983,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>350</v>
       </c>
@@ -4014,7 +4000,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>353</v>
       </c>
@@ -4031,7 +4017,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>356</v>
       </c>
@@ -4048,7 +4034,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>358</v>
       </c>
@@ -4065,7 +4051,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>361</v>
       </c>
@@ -4082,7 +4068,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>363</v>
       </c>
@@ -4099,7 +4085,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>366</v>
       </c>
@@ -4116,7 +4102,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>368</v>
       </c>
@@ -4133,7 +4119,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>371</v>
       </c>
@@ -4150,7 +4136,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>374</v>
       </c>
@@ -4167,7 +4153,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>378</v>
       </c>
@@ -4184,7 +4170,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>381</v>
       </c>
@@ -4201,7 +4187,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>383</v>
       </c>
@@ -4218,7 +4204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>385</v>
       </c>
@@ -4235,7 +4221,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>387</v>
       </c>
@@ -4252,7 +4238,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>389</v>
       </c>
@@ -4269,7 +4255,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>392</v>
       </c>
@@ -4286,7 +4272,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>395</v>
       </c>
@@ -4303,7 +4289,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>397</v>
       </c>
@@ -4320,7 +4306,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>399</v>
       </c>
@@ -4337,7 +4323,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>401</v>
       </c>
@@ -4354,7 +4340,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>403</v>
       </c>
@@ -4371,7 +4357,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>406</v>
       </c>
@@ -4388,7 +4374,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>408</v>
       </c>
@@ -4405,7 +4391,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>411</v>
       </c>
@@ -4422,7 +4408,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>413</v>
       </c>
@@ -4439,7 +4425,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>416</v>
       </c>
@@ -4456,7 +4442,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>418</v>
       </c>
@@ -4473,7 +4459,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>420</v>
       </c>
@@ -4490,7 +4476,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>423</v>
       </c>
@@ -4507,7 +4493,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>426</v>
       </c>
@@ -4524,7 +4510,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>429</v>
       </c>
@@ -4541,7 +4527,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>431</v>
       </c>
@@ -4558,7 +4544,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>434</v>
       </c>
@@ -4575,7 +4561,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>436</v>
       </c>
@@ -4592,7 +4578,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>438</v>
       </c>
@@ -4609,7 +4595,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>441</v>
       </c>
@@ -4626,7 +4612,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>443</v>
       </c>
@@ -4643,7 +4629,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>446</v>
       </c>
@@ -4660,7 +4646,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>448</v>
       </c>
@@ -4677,7 +4663,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>450</v>
       </c>
@@ -4694,7 +4680,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>453</v>
       </c>
@@ -4711,7 +4697,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>455</v>
       </c>
@@ -4728,7 +4714,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>458</v>
       </c>
@@ -4745,7 +4731,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>460</v>
       </c>
@@ -4762,7 +4748,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>463</v>
       </c>
@@ -4779,7 +4765,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>465</v>
       </c>
@@ -4796,7 +4782,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>468</v>
       </c>
@@ -4813,7 +4799,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>471</v>
       </c>
@@ -4830,7 +4816,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>473</v>
       </c>
@@ -4847,7 +4833,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>418</v>
       </c>
@@ -4864,7 +4850,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>477</v>
       </c>
@@ -4881,7 +4867,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>480</v>
       </c>
@@ -4898,7 +4884,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>482</v>
       </c>
@@ -4915,7 +4901,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>484</v>
       </c>
@@ -4932,7 +4918,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>486</v>
       </c>
@@ -4949,7 +4935,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>489</v>
       </c>
@@ -4966,7 +4952,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>491</v>
       </c>
@@ -4983,7 +4969,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>494</v>
       </c>
@@ -5000,7 +4986,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" s="4" t="s">
         <v>513</v>
       </c>
@@ -5017,7 +5003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" s="5">
         <v>336</v>
       </c>
@@ -5034,7 +5020,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" s="5">
         <v>5</v>
       </c>
@@ -5051,7 +5037,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" s="6">
         <v>337</v>
       </c>
@@ -5068,7 +5054,7 @@
         <v>122103</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" s="6">
         <v>338</v>
       </c>
@@ -5085,7 +5071,7 @@
         <v>140417</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A179" s="6">
         <v>340</v>
       </c>
@@ -5102,7 +5088,7 @@
         <v>501510</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A180" s="6">
         <v>339</v>
       </c>
@@ -5119,7 +5105,7 @@
         <v>501401</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A181" s="6">
         <v>346</v>
       </c>
@@ -5136,7 +5122,7 @@
         <v>493221</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A182" s="6">
         <v>341</v>
       </c>
@@ -5153,7 +5139,7 @@
         <v>781122</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A183" s="6">
         <v>345</v>
       </c>
@@ -5170,7 +5156,7 @@
         <v>711322</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A184" s="6">
         <v>344</v>
       </c>
@@ -5187,7 +5173,7 @@
         <v>226401</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A185" s="6">
         <v>342</v>
       </c>
@@ -5204,7 +5190,7 @@
         <v>752054</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A186" s="6">
         <v>343</v>
       </c>
@@ -5221,7 +5207,7 @@
         <v>804451</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A187" s="7">
         <v>347</v>
       </c>
@@ -5238,7 +5224,7 @@
         <v>600067</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A188" s="7">
         <v>348</v>
       </c>
@@ -5255,7 +5241,7 @@
         <v>387540</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A189" s="7">
         <v>349</v>
       </c>
@@ -5272,7 +5258,7 @@
         <v>209859</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A190" s="7">
         <v>350</v>
       </c>
@@ -5289,7 +5275,7 @@
         <v>122506</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A191" s="7">
         <v>1003</v>
       </c>
@@ -5306,7 +5292,7 @@
         <v>421302</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A192" s="7">
         <v>351</v>
       </c>
@@ -5323,7 +5309,7 @@
         <v>500034</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A193" s="7">
         <v>352</v>
       </c>
@@ -5338,23 +5324,6 @@
       </c>
       <c r="E193" s="6">
         <v>712223</v>
-      </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A194" s="7">
-        <v>353</v>
-      </c>
-      <c r="B194" s="1" t="s">
-        <v>512</v>
-      </c>
-      <c r="C194" s="6" t="s">
-        <v>536</v>
-      </c>
-      <c r="D194" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="E194" s="6">
-        <v>641402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>